<commit_message>
Initial commit - AIExcelLogger project
</commit_message>
<xml_diff>
--- a/worklog.xlsx
+++ b/worklog.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="46">
   <si>
     <t>Date</t>
   </si>
@@ -115,6 +115,66 @@
   </si>
   <si>
     <t>false</t>
+  </si>
+  <si>
+    <t>• Worked on SailPoint custom connector creation for MySQL.</t>
+  </si>
+  <si>
+    <t>• Designed and developed a custom SailPoint connector to integrate with MySQL, enabling seamless data synchronization between the two platforms.
+• Implemented robust error handling mechanisms to ensure reliable data transfer.
+• Conducted thorough testing to validate the connector's functionality and performance.</t>
+  </si>
+  <si>
+    <t>• Designed and developed a custom connector for SailPoint to integrate with MySQL, ensuring seamless data exchange.
+• Implemented robust error handling and logging mechanisms to ensure reliable connectivity.
+• Conducted thorough testing to guarantee compatibility with various MySQL versions and configurations.</t>
+  </si>
+  <si>
+    <t>2026-03-23</t>
+  </si>
+  <si>
+    <t>Detailed explanation here</t>
+  </si>
+  <si>
+    <t>Sailpoint Custom Workflow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+• Worked on sailpoint custom workflow for JML
+• Attended a meeting with client</t>
+  </si>
+  <si>
+    <t>saviynt</t>
+  </si>
+  <si>
+    <t>• created JML process
+• attended standup call</t>
+  </si>
+  <si>
+    <t>1) Created JML process for saviynt, defining technical rules to ensure efficient processing.
+2) Attended standup call to discuss ongoing projects and goals, ensuring alignment with team objectives.</t>
+  </si>
+  <si>
+    <t>continue working on JML process</t>
+  </si>
+  <si>
+    <t>2026-03-29</t>
+  </si>
+  <si>
+    <t>Saviynt Custom Certification</t>
+  </si>
+  <si>
+    <t>• Created a custom application owner certificate
+• Helped Shubhangini with the certification process
+• Attended stand-up call</t>
+  </si>
+  <si>
+    <t>1) Created a custom application owner certificate to enhance the certification process, which was done by following the Saviynt guidelines and using the available tools, and this was necessary to improve the overall certification experience. 
+2) Helped Shubhangini with the certification process by providing guidance and support, which was done through a collaborative approach and open communication, and this was necessary to ensure that she had a clear understanding of the process. 
+3) Attended the stand-up call to discuss the project's progress and address any concerns, which was done by actively participating in the discussion and providing updates on my tasks, and this was necessary to ensure that everyone was on the same page and that the project was moving forward as planned.</t>
+  </si>
+  <si>
+    <t>Continue working on the Saviynt custom certification project</t>
   </si>
 </sst>
 </file>
@@ -151,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment wrapText="true"/>
@@ -167,6 +227,27 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment wrapText="true" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment wrapText="true" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment wrapText="true" vertical="top"/>
     </xf>
   </cellXfs>
 </styleSheet>
@@ -174,15 +255,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="10.13671875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="16.49609375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="23.60546875"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="52.609375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="209.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="247.1953125"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="15.2734375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="18.3828125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="49.625"/>
     <col min="7" max="7" bestFit="true" customWidth="true" width="9.80078125"/>
     <col min="8" max="8" bestFit="true" customWidth="true" width="8.41015625"/>
     <col min="9" max="9" bestFit="true" customWidth="true" width="11.1484375"/>
@@ -381,6 +462,206 @@
         <v>14</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s" s="6">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s" s="6">
+        <v>31</v>
+      </c>
+      <c r="E7" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="F7" s="0"/>
+      <c r="G7" s="0"/>
+      <c r="H7" s="0"/>
+      <c r="I7" s="0"/>
+      <c r="J7" s="0"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="C8" t="s" s="7">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s" s="7">
+        <v>32</v>
+      </c>
+      <c r="E8" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="F8" s="0"/>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
+      <c r="I8" s="0"/>
+      <c r="J8" s="0"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" t="s" s="8">
+        <v>34</v>
+      </c>
+      <c r="E9" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="G9" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="I9" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="J9" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C10" s="9"/>
+      <c r="D10" t="s" s="9">
+        <v>14</v>
+      </c>
+      <c r="E10" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="G10" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="I10" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="J10" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s" s="10">
+        <v>36</v>
+      </c>
+      <c r="D11" t="s" s="10">
+        <v>34</v>
+      </c>
+      <c r="E11" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="F11" t="s" s="10">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="H11" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="I11" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="J11" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="C12" t="s" s="11">
+        <v>38</v>
+      </c>
+      <c r="D12" t="s" s="11">
+        <v>39</v>
+      </c>
+      <c r="E12" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="F12" t="s" s="11">
+        <v>40</v>
+      </c>
+      <c r="G12" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="H12" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="I12" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="J12" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C13" t="s" s="12">
+        <v>43</v>
+      </c>
+      <c r="D13" t="s" s="12">
+        <v>44</v>
+      </c>
+      <c r="E13" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="F13" t="s" s="12">
+        <v>45</v>
+      </c>
+      <c r="G13" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="H13" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="I13" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="J13" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>